<commit_message>
rationalisation improved - dynamic batch sizes
</commit_message>
<xml_diff>
--- a/sample_data/OrgSight_Sample_OrgChart_28rows.xlsx
+++ b/sample_data/OrgSight_Sample_OrgChart_28rows.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itinfoalvarezandmarsalind-my.sharepoint.com/personal/jagritjain_alvarezandmarsal_com/Documents/Documents/APPS/ORG_ANALYSIS/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_F9A1AFDACB6FCA12B72D4C3E9D07A8864FA89CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D07FE555-AE11-40DA-967E-64B366011B7A}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_F9A1AFDACB6FCA12B72D4C3E9D07A8864FA89CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8537177-0E0D-455E-8959-AA01F075F80B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4800" yWindow="3290" windowWidth="14400" windowHeight="8710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Census" sheetId="1" r:id="rId1"/>
@@ -817,6 +817,11 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="27.7265625" customWidth="1"/>
+    <col min="5" max="5" width="34.90625" customWidth="1"/>
+    <col min="6" max="6" width="30.7265625" customWidth="1"/>
+    <col min="7" max="7" width="37.36328125" customWidth="1"/>
+    <col min="8" max="8" width="31.6328125" customWidth="1"/>
     <col min="10" max="10" width="19.453125" customWidth="1"/>
     <col min="11" max="11" width="25.81640625" customWidth="1"/>
   </cols>

</xml_diff>